<commit_message>
A few updates to replacement data
</commit_message>
<xml_diff>
--- a/Trees/STO/Replacement tracking/Tree replacements.xlsx
+++ b/Trees/STO/Replacement tracking/Tree replacements.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11110"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10526"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kent/Dev/Noho/Trees/STO/Replacement tracking/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F684CDF-CC53-EF40-B4CD-EEDE78E21E29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{217F388A-0A14-F341-84F8-E69EFE9C4386}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10120" yWindow="2780" windowWidth="34360" windowHeight="16580" xr2:uid="{B7658DB7-84F7-914E-8320-8DBFC49D6E54}"/>
+    <workbookView xWindow="4820" yWindow="1400" windowWidth="30620" windowHeight="21820" xr2:uid="{B7658DB7-84F7-914E-8320-8DBFC49D6E54}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="172" uniqueCount="140">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="175" uniqueCount="144">
   <si>
     <t>Permit</t>
   </si>
@@ -245,18 +245,12 @@
     <t>Planning Board 40R</t>
   </si>
   <si>
-    <t>Bridge St</t>
-  </si>
-  <si>
     <t>Valley CDC</t>
   </si>
   <si>
     <t>Zoning Board of Appeals Spec. Permit</t>
   </si>
   <si>
-    <t>Prospect St</t>
-  </si>
-  <si>
     <t>Nields-Duffy</t>
   </si>
   <si>
@@ -456,6 +450,24 @@
   </si>
   <si>
     <t>21 Olander Dr</t>
+  </si>
+  <si>
+    <t>82 Bridge St</t>
+  </si>
+  <si>
+    <t>32A-178-001</t>
+  </si>
+  <si>
+    <t>415 Prospect St</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 24A-103-001</t>
+  </si>
+  <si>
+    <t>88 Village Hill</t>
+  </si>
+  <si>
+    <t>31C-047-003</t>
   </si>
 </sst>
 </file>
@@ -870,7 +882,7 @@
         <v>2</v>
       </c>
       <c r="D1" s="6" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="E1" s="6" t="s">
         <v>3</v>
@@ -891,7 +903,7 @@
         <v>32</v>
       </c>
       <c r="K1" s="6" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="L1" s="6" t="s">
         <v>33</v>
@@ -914,7 +926,7 @@
         <v>6</v>
       </c>
       <c r="D2" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="E2" t="s">
         <v>7</v>
@@ -943,7 +955,7 @@
         <v>9</v>
       </c>
       <c r="D3" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="E3" t="s">
         <v>10</v>
@@ -975,7 +987,7 @@
         <v>12</v>
       </c>
       <c r="D4" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="E4" t="s">
         <v>13</v>
@@ -1010,7 +1022,7 @@
         <v>14</v>
       </c>
       <c r="D5" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="E5" t="s">
         <v>15</v>
@@ -1042,7 +1054,7 @@
         <v>17</v>
       </c>
       <c r="D6" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="E6" t="s">
         <v>18</v>
@@ -1077,7 +1089,7 @@
         <v>19</v>
       </c>
       <c r="D7" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="E7" t="s">
         <v>20</v>
@@ -1112,7 +1124,7 @@
         <v>12</v>
       </c>
       <c r="D8" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="E8" t="s">
         <v>22</v>
@@ -1147,7 +1159,7 @@
         <v>23</v>
       </c>
       <c r="D9" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="E9" t="s">
         <v>24</v>
@@ -1179,7 +1191,7 @@
         <v>25</v>
       </c>
       <c r="D10" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="E10" t="s">
         <v>26</v>
@@ -1211,7 +1223,7 @@
         <v>27</v>
       </c>
       <c r="D11" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="E11" t="s">
         <v>28</v>
@@ -1246,7 +1258,7 @@
         <v>42</v>
       </c>
       <c r="D12" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="E12" t="s">
         <v>43</v>
@@ -1275,10 +1287,10 @@
         <v>42491</v>
       </c>
       <c r="C13" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="D13" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="E13" t="s">
         <v>45</v>
@@ -1316,10 +1328,10 @@
         <v>47</v>
       </c>
       <c r="D14" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="E14" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="F14">
         <v>14</v>
@@ -1348,7 +1360,7 @@
         <v>49</v>
       </c>
       <c r="D15" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="E15" t="s">
         <v>50</v>
@@ -1383,7 +1395,7 @@
         <v>52</v>
       </c>
       <c r="E16" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="F16">
         <v>1</v>
@@ -1412,10 +1424,10 @@
         <v>42552</v>
       </c>
       <c r="C17" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="D17" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="E17" t="s">
         <v>54</v>
@@ -1447,10 +1459,10 @@
         <v>42614</v>
       </c>
       <c r="C18" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="D18" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="E18" t="s">
         <v>56</v>
@@ -1488,10 +1500,10 @@
         <v>44317</v>
       </c>
       <c r="C19" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="D19" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="E19" t="s">
         <v>58</v>
@@ -1512,7 +1524,7 @@
         <v>2100</v>
       </c>
       <c r="N19" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
     </row>
     <row r="20" spans="1:14" x14ac:dyDescent="0.2">
@@ -1526,7 +1538,7 @@
         <v>59</v>
       </c>
       <c r="D20" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="E20" t="s">
         <v>60</v>
@@ -1555,10 +1567,10 @@
         <v>42767</v>
       </c>
       <c r="C21" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="D21" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="E21" t="s">
         <v>61</v>
@@ -1636,10 +1648,10 @@
         <v>42887</v>
       </c>
       <c r="C24" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="E24" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="F24">
         <v>1</v>
@@ -1661,10 +1673,13 @@
         <v>42948</v>
       </c>
       <c r="C25" t="s">
+        <v>138</v>
+      </c>
+      <c r="D25" t="s">
+        <v>139</v>
+      </c>
+      <c r="E25" t="s">
         <v>69</v>
-      </c>
-      <c r="E25" t="s">
-        <v>70</v>
       </c>
       <c r="F25">
         <v>4</v>
@@ -1676,27 +1691,30 @@
         <v>600</v>
       </c>
       <c r="L25" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="M25">
         <v>600</v>
       </c>
       <c r="N25" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
     </row>
     <row r="26" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B26" s="3">
         <v>42948</v>
       </c>
       <c r="C26" t="s">
-        <v>72</v>
+        <v>140</v>
+      </c>
+      <c r="D26" t="s">
+        <v>141</v>
       </c>
       <c r="E26" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="F26">
         <v>2</v>
@@ -1719,10 +1737,13 @@
         <v>42979</v>
       </c>
       <c r="C27" t="s">
-        <v>47</v>
+        <v>142</v>
+      </c>
+      <c r="D27" t="s">
+        <v>143</v>
       </c>
       <c r="E27" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="F27">
         <v>1</v>
@@ -1737,21 +1758,21 @@
         <v>5</v>
       </c>
       <c r="N27" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
     </row>
     <row r="28" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="B28" s="3">
         <v>42614</v>
       </c>
       <c r="C28" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="E28" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="F28">
         <v>16</v>
@@ -1765,30 +1786,30 @@
     </row>
     <row r="29" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="B29" s="3">
         <v>42614</v>
       </c>
       <c r="C29" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="E29" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
     </row>
     <row r="30" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="B30" s="3">
         <v>43009</v>
       </c>
       <c r="C30" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="E30" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="F30">
         <v>30</v>
@@ -1809,12 +1830,12 @@
         <v>30900</v>
       </c>
       <c r="N30" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
     </row>
     <row r="31" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="B31" s="3">
         <v>43435</v>
@@ -1823,7 +1844,7 @@
         <v>63</v>
       </c>
       <c r="E31" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="F31">
         <v>247</v>
@@ -1841,7 +1862,7 @@
         <v>318800</v>
       </c>
       <c r="N31" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
     </row>
     <row r="32" spans="1:14" x14ac:dyDescent="0.2">
@@ -1852,10 +1873,10 @@
         <v>43405</v>
       </c>
       <c r="C32" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="E32" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="F32">
         <v>80</v>
@@ -1876,21 +1897,21 @@
         <v>86000</v>
       </c>
       <c r="N32" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
     </row>
     <row r="33" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="B33" s="3">
         <v>43374</v>
       </c>
       <c r="C33" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="E33" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="F33">
         <v>20</v>
@@ -1905,21 +1926,21 @@
         <v>110</v>
       </c>
       <c r="N33" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
     </row>
     <row r="34" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="B34" s="3">
         <v>43344</v>
       </c>
       <c r="C34" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="E34" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="F34">
         <v>1</v>
@@ -1934,21 +1955,21 @@
         <v>6</v>
       </c>
       <c r="N34" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
     </row>
     <row r="35" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="B35" s="3">
         <v>43101</v>
       </c>
       <c r="C35" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="E35" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="F35">
         <v>15</v>
@@ -1963,7 +1984,7 @@
         <v>86</v>
       </c>
       <c r="N35" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
     </row>
     <row r="36" spans="1:14" x14ac:dyDescent="0.2">
@@ -1974,10 +1995,10 @@
         <v>43617</v>
       </c>
       <c r="C36" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="E36" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="F36">
         <v>9</v>
@@ -1989,7 +2010,7 @@
         <v>70</v>
       </c>
       <c r="N36" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
     </row>
     <row r="37" spans="1:14" x14ac:dyDescent="0.2">
@@ -2000,10 +2021,10 @@
         <v>43525</v>
       </c>
       <c r="C37" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="E37" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="F37">
         <v>2</v>
@@ -2024,7 +2045,7 @@
         <v>750</v>
       </c>
       <c r="N37" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
     </row>
     <row r="38" spans="1:14" x14ac:dyDescent="0.2">
@@ -2035,10 +2056,10 @@
         <v>44256</v>
       </c>
       <c r="C38" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="E38" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="F38">
         <v>5</v>
@@ -2047,7 +2068,7 @@
         <v>108</v>
       </c>
       <c r="H38" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="K38" s="4">
         <v>3200</v>
@@ -2059,7 +2080,7 @@
         <v>3200</v>
       </c>
       <c r="N38" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
     </row>
     <row r="39" spans="1:14" x14ac:dyDescent="0.2">
@@ -2067,10 +2088,10 @@
         <v>48</v>
       </c>
       <c r="C39" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="E39" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="F39">
         <v>2</v>

</xml_diff>